<commit_message>
Ajustando cambios en accesos para seguridad
</commit_message>
<xml_diff>
--- a/public/plantillas/2026_INFORME_SEGURIDAD.xlsx
+++ b/public/plantillas/2026_INFORME_SEGURIDAD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5D6026-0948-E144-B563-00ACC708F493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88871DF7-4CF8-7747-BC84-37E67455FD7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Table 1'!$A$1:$F$29</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Table 2'!$A$1:$M$39</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Table 3'!$A$1:$K$99</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Table 3'!$A$1:$K$100</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="111">
   <si>
     <t>Rehabilitación, Sustitución y/o Modernización de 526 puentes  de la Línea K ixtepec, Oax. - C.D Hidalgo, Chiapas y KA  los toros-Puerto  Chiapas referente al Programa  para el Desarrollo del Istmo  de Tehuantepec 2020-2024</t>
   </si>
@@ -459,6 +459,12 @@
   </si>
   <si>
     <t>Guzman Aguirre Asaf</t>
+  </si>
+  <si>
+    <t>Personal rotativo durante el periodo</t>
+  </si>
+  <si>
+    <t>Personal administrativo</t>
   </si>
 </sst>
 </file>
@@ -1687,7 +1693,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="235">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2051,42 +2057,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2099,15 +2084,102 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2117,24 +2189,6 @@
     <xf numFmtId="1" fontId="15" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2144,52 +2198,154 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2240,156 +2396,7 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2930,73 +2937,73 @@
       <c r="E4" s="1"/>
     </row>
     <row r="7" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B7" s="121" t="s">
+      <c r="B7" s="123" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="128"/>
-      <c r="D7" s="128"/>
-      <c r="E7" s="129"/>
+      <c r="C7" s="124"/>
+      <c r="D7" s="124"/>
+      <c r="E7" s="125"/>
     </row>
     <row r="8" spans="2:5" ht="34.5" customHeight="1">
       <c r="B8" s="4" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="131" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="132"/>
+      <c r="D8" s="121" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="122"/>
     </row>
     <row r="9" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B9" s="133" t="s">
+      <c r="B9" s="126" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="132"/>
+      <c r="C9" s="122"/>
       <c r="D9" s="104" t="s">
         <v>1</v>
       </c>
       <c r="E9" s="105"/>
     </row>
     <row r="10" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B10" s="133" t="s">
+      <c r="B10" s="126" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="132"/>
-      <c r="D10" s="134"/>
-      <c r="E10" s="134"/>
+      <c r="C10" s="122"/>
+      <c r="D10" s="127"/>
+      <c r="E10" s="127"/>
     </row>
     <row r="11" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B11" s="133" t="s">
+      <c r="B11" s="126" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="132"/>
-      <c r="D11" s="134"/>
-      <c r="E11" s="134"/>
+      <c r="C11" s="122"/>
+      <c r="D11" s="127"/>
+      <c r="E11" s="127"/>
     </row>
     <row r="12" spans="2:5" ht="16.25" customHeight="1">
-      <c r="B12" s="133" t="s">
+      <c r="B12" s="126" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="132"/>
-      <c r="D12" s="135"/>
-      <c r="E12" s="136"/>
+      <c r="C12" s="122"/>
+      <c r="D12" s="128"/>
+      <c r="E12" s="129"/>
     </row>
     <row r="13" spans="2:5" ht="19.25" customHeight="1">
-      <c r="B13" s="121" t="s">
+      <c r="B13" s="123" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="122"/>
-      <c r="D13" s="122"/>
-      <c r="E13" s="123"/>
+      <c r="C13" s="130"/>
+      <c r="D13" s="130"/>
+      <c r="E13" s="131"/>
     </row>
     <row r="14" spans="2:5" ht="16.5" customHeight="1">
       <c r="B14" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="124" t="s">
+      <c r="C14" s="132" t="s">
         <v>4</v>
       </c>
-      <c r="D14" s="124"/>
+      <c r="D14" s="132"/>
       <c r="E14" s="103" t="s">
         <v>3</v>
       </c>
@@ -3038,12 +3045,12 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="18" customHeight="1">
-      <c r="B18" s="130" t="s">
+      <c r="B18" s="136" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="128"/>
-      <c r="D18" s="128"/>
-      <c r="E18" s="123"/>
+      <c r="C18" s="124"/>
+      <c r="D18" s="124"/>
+      <c r="E18" s="131"/>
       <c r="H18" s="3" t="s">
         <v>10</v>
       </c>
@@ -3052,10 +3059,10 @@
       <c r="B19" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="125" t="s">
+      <c r="C19" s="133" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="126"/>
+      <c r="D19" s="134"/>
       <c r="E19" s="8" t="s">
         <v>3</v>
       </c>
@@ -3069,21 +3076,21 @@
       <c r="E20" s="9"/>
     </row>
     <row r="21" spans="2:8" ht="17.25" customHeight="1">
-      <c r="B21" s="121" t="s">
+      <c r="B21" s="123" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="128"/>
-      <c r="D21" s="128"/>
-      <c r="E21" s="129"/>
+      <c r="C21" s="124"/>
+      <c r="D21" s="124"/>
+      <c r="E21" s="125"/>
     </row>
     <row r="22" spans="2:8" ht="17.25" customHeight="1">
       <c r="B22" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C22" s="125" t="s">
+      <c r="C22" s="133" t="s">
         <v>4</v>
       </c>
-      <c r="D22" s="126"/>
+      <c r="D22" s="134"/>
       <c r="E22" s="8" t="s">
         <v>3</v>
       </c>
@@ -3101,21 +3108,21 @@
       </c>
     </row>
     <row r="24" spans="2:8">
-      <c r="B24" s="127" t="s">
+      <c r="B24" s="135" t="s">
         <v>16</v>
       </c>
-      <c r="C24" s="128"/>
-      <c r="D24" s="128"/>
-      <c r="E24" s="129"/>
+      <c r="C24" s="124"/>
+      <c r="D24" s="124"/>
+      <c r="E24" s="125"/>
     </row>
     <row r="25" spans="2:8" ht="14">
       <c r="B25" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="125" t="s">
+      <c r="C25" s="133" t="s">
         <v>4</v>
       </c>
-      <c r="D25" s="126"/>
+      <c r="D25" s="134"/>
       <c r="E25" s="8" t="s">
         <v>3</v>
       </c>
@@ -3130,6 +3137,14 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="B21:E21"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="B10:C10"/>
@@ -3139,14 +3154,6 @@
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="B21:E21"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -3219,47 +3226,47 @@
       <c r="L3" s="13"/>
     </row>
     <row r="4" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B4" s="143" t="s">
+      <c r="B4" s="155" t="s">
         <v>92</v>
       </c>
-      <c r="C4" s="144"/>
-      <c r="D4" s="144"/>
-      <c r="E4" s="144"/>
-      <c r="F4" s="144"/>
-      <c r="G4" s="144"/>
-      <c r="H4" s="144"/>
-      <c r="I4" s="144"/>
-      <c r="J4" s="144"/>
-      <c r="K4" s="144"/>
-      <c r="L4" s="145"/>
+      <c r="C4" s="156"/>
+      <c r="D4" s="156"/>
+      <c r="E4" s="156"/>
+      <c r="F4" s="156"/>
+      <c r="G4" s="156"/>
+      <c r="H4" s="156"/>
+      <c r="I4" s="156"/>
+      <c r="J4" s="156"/>
+      <c r="K4" s="156"/>
+      <c r="L4" s="157"/>
       <c r="M4" s="70"/>
       <c r="N4" s="70"/>
       <c r="O4" s="70"/>
     </row>
     <row r="5" spans="2:15" ht="18" customHeight="1">
-      <c r="B5" s="146" t="s">
+      <c r="B5" s="158" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="147"/>
-      <c r="D5" s="147"/>
-      <c r="E5" s="147"/>
-      <c r="F5" s="147"/>
-      <c r="G5" s="147"/>
-      <c r="H5" s="147"/>
-      <c r="I5" s="147"/>
-      <c r="J5" s="147"/>
-      <c r="K5" s="147"/>
-      <c r="L5" s="148"/>
+      <c r="C5" s="159"/>
+      <c r="D5" s="159"/>
+      <c r="E5" s="159"/>
+      <c r="F5" s="159"/>
+      <c r="G5" s="159"/>
+      <c r="H5" s="159"/>
+      <c r="I5" s="159"/>
+      <c r="J5" s="159"/>
+      <c r="K5" s="159"/>
+      <c r="L5" s="160"/>
       <c r="M5" s="71"/>
       <c r="N5" s="71"/>
       <c r="O5" s="71"/>
     </row>
     <row r="6" spans="2:15" ht="30" customHeight="1">
-      <c r="B6" s="149" t="s">
+      <c r="B6" s="165" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="150"/>
-      <c r="D6" s="151"/>
+      <c r="C6" s="166"/>
+      <c r="D6" s="167"/>
       <c r="E6" s="72" t="s">
         <v>19</v>
       </c>
@@ -3286,10 +3293,10 @@
       </c>
     </row>
     <row r="7" spans="2:15" ht="18.75" customHeight="1">
-      <c r="B7" s="137" t="s">
+      <c r="B7" s="141" t="s">
         <v>104</v>
       </c>
-      <c r="C7" s="138"/>
+      <c r="C7" s="161"/>
       <c r="D7" s="87" t="s">
         <v>98</v>
       </c>
@@ -3314,14 +3321,14 @@
       <c r="K7" s="88">
         <v>0</v>
       </c>
-      <c r="L7" s="141">
+      <c r="L7" s="163">
         <f>SUM(E8:I8)*10+(J8*J7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:15" ht="18.75" customHeight="1">
-      <c r="B8" s="139"/>
-      <c r="C8" s="140"/>
+      <c r="B8" s="147"/>
+      <c r="C8" s="162"/>
       <c r="D8" s="76" t="s">
         <v>99</v>
       </c>
@@ -3346,13 +3353,13 @@
       <c r="K8" s="74">
         <v>0</v>
       </c>
-      <c r="L8" s="142"/>
+      <c r="L8" s="164"/>
     </row>
     <row r="9" spans="2:15" ht="18" customHeight="1">
-      <c r="B9" s="137" t="s">
+      <c r="B9" s="141" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="138"/>
+      <c r="C9" s="161"/>
       <c r="D9" s="87" t="s">
         <v>98</v>
       </c>
@@ -3377,14 +3384,14 @@
       <c r="K9" s="88">
         <v>0</v>
       </c>
-      <c r="L9" s="141">
+      <c r="L9" s="163">
         <f>SUM(E10:I10)*10+(J10*J9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="2:15" ht="18" customHeight="1">
-      <c r="B10" s="139"/>
-      <c r="C10" s="140"/>
+      <c r="B10" s="147"/>
+      <c r="C10" s="162"/>
       <c r="D10" s="76" t="s">
         <v>99</v>
       </c>
@@ -3409,13 +3416,13 @@
       <c r="K10" s="74">
         <v>0</v>
       </c>
-      <c r="L10" s="142"/>
+      <c r="L10" s="164"/>
     </row>
     <row r="11" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B11" s="137" t="s">
+      <c r="B11" s="141" t="s">
         <v>104</v>
       </c>
-      <c r="C11" s="138"/>
+      <c r="C11" s="161"/>
       <c r="D11" s="87" t="s">
         <v>98</v>
       </c>
@@ -3440,14 +3447,14 @@
       <c r="K11" s="88">
         <v>0</v>
       </c>
-      <c r="L11" s="141">
+      <c r="L11" s="163">
         <f>SUM(E12:I12)*10+(J12*J11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B12" s="139"/>
-      <c r="C12" s="140"/>
+      <c r="B12" s="147"/>
+      <c r="C12" s="162"/>
       <c r="D12" s="76" t="s">
         <v>99</v>
       </c>
@@ -3472,13 +3479,13 @@
       <c r="K12" s="74">
         <v>0</v>
       </c>
-      <c r="L12" s="142"/>
+      <c r="L12" s="164"/>
     </row>
     <row r="13" spans="2:15" ht="18" customHeight="1">
-      <c r="B13" s="137" t="s">
+      <c r="B13" s="141" t="s">
         <v>104</v>
       </c>
-      <c r="C13" s="138"/>
+      <c r="C13" s="161"/>
       <c r="D13" s="87" t="s">
         <v>98</v>
       </c>
@@ -3503,14 +3510,14 @@
       <c r="K13" s="88">
         <v>0</v>
       </c>
-      <c r="L13" s="141">
+      <c r="L13" s="163">
         <f>SUM(E14:I14)*10+(J14*J13)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:15" ht="18" customHeight="1">
-      <c r="B14" s="139"/>
-      <c r="C14" s="140"/>
+      <c r="B14" s="147"/>
+      <c r="C14" s="162"/>
       <c r="D14" s="76" t="s">
         <v>99</v>
       </c>
@@ -3535,13 +3542,13 @@
       <c r="K14" s="74">
         <v>0</v>
       </c>
-      <c r="L14" s="142"/>
+      <c r="L14" s="164"/>
     </row>
     <row r="15" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B15" s="137" t="s">
+      <c r="B15" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C15" s="138"/>
+      <c r="C15" s="161"/>
       <c r="D15" s="87" t="s">
         <v>98</v>
       </c>
@@ -3566,14 +3573,14 @@
       <c r="K15" s="88">
         <v>0</v>
       </c>
-      <c r="L15" s="141">
+      <c r="L15" s="163">
         <f>SUM(E16:I16)*10+(J16*J15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B16" s="139"/>
-      <c r="C16" s="140"/>
+      <c r="B16" s="147"/>
+      <c r="C16" s="162"/>
       <c r="D16" s="76" t="s">
         <v>99</v>
       </c>
@@ -3598,13 +3605,13 @@
       <c r="K16" s="74">
         <v>0</v>
       </c>
-      <c r="L16" s="142"/>
+      <c r="L16" s="164"/>
     </row>
     <row r="17" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B17" s="137" t="s">
+      <c r="B17" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C17" s="138"/>
+      <c r="C17" s="161"/>
       <c r="D17" s="87" t="s">
         <v>98</v>
       </c>
@@ -3629,14 +3636,14 @@
       <c r="K17" s="88">
         <v>0</v>
       </c>
-      <c r="L17" s="141">
+      <c r="L17" s="163">
         <f>SUM(E18:I18)*10+(J18*J17)</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B18" s="139"/>
-      <c r="C18" s="140"/>
+      <c r="B18" s="147"/>
+      <c r="C18" s="162"/>
       <c r="D18" s="76" t="s">
         <v>99</v>
       </c>
@@ -3661,13 +3668,13 @@
       <c r="K18" s="74">
         <v>0</v>
       </c>
-      <c r="L18" s="142"/>
+      <c r="L18" s="164"/>
     </row>
     <row r="19" spans="2:15" ht="18" customHeight="1">
-      <c r="B19" s="137" t="s">
+      <c r="B19" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C19" s="138"/>
+      <c r="C19" s="161"/>
       <c r="D19" s="87" t="s">
         <v>98</v>
       </c>
@@ -3692,14 +3699,14 @@
       <c r="K19" s="88">
         <v>0</v>
       </c>
-      <c r="L19" s="141">
+      <c r="L19" s="163">
         <f>SUM(E20:I20)*10+(J20*J19)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="2:15" ht="18" customHeight="1">
-      <c r="B20" s="139"/>
-      <c r="C20" s="140"/>
+      <c r="B20" s="147"/>
+      <c r="C20" s="162"/>
       <c r="D20" s="76" t="s">
         <v>99</v>
       </c>
@@ -3724,13 +3731,13 @@
       <c r="K20" s="74">
         <v>0</v>
       </c>
-      <c r="L20" s="142"/>
+      <c r="L20" s="164"/>
     </row>
     <row r="21" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B21" s="137" t="s">
+      <c r="B21" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C21" s="138"/>
+      <c r="C21" s="161"/>
       <c r="D21" s="87" t="s">
         <v>98</v>
       </c>
@@ -3755,14 +3762,14 @@
       <c r="K21" s="88">
         <v>0</v>
       </c>
-      <c r="L21" s="141">
+      <c r="L21" s="163">
         <f>SUM(E22:I22)*10+(J22*J21)</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B22" s="139"/>
-      <c r="C22" s="140"/>
+      <c r="B22" s="147"/>
+      <c r="C22" s="162"/>
       <c r="D22" s="76" t="s">
         <v>99</v>
       </c>
@@ -3787,14 +3794,14 @@
       <c r="K22" s="74">
         <v>0</v>
       </c>
-      <c r="L22" s="142"/>
+      <c r="L22" s="164"/>
     </row>
     <row r="23" spans="2:15" ht="18" customHeight="1">
-      <c r="B23" s="156" t="s">
+      <c r="B23" s="149" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="157"/>
-      <c r="D23" s="158"/>
+      <c r="C23" s="150"/>
+      <c r="D23" s="151"/>
       <c r="E23" s="85">
         <f>SUM(E8,E10,E12,E14,E16,E18,E20,E22)</f>
         <v>0</v>
@@ -3841,28 +3848,28 @@
       <c r="K24" s="75"/>
     </row>
     <row r="25" spans="2:15" ht="15" customHeight="1">
-      <c r="B25" s="163" t="s">
+      <c r="B25" s="154" t="s">
         <v>94</v>
       </c>
-      <c r="C25" s="163"/>
-      <c r="D25" s="163"/>
-      <c r="E25" s="163"/>
-      <c r="F25" s="163"/>
-      <c r="G25" s="163"/>
-      <c r="H25" s="163"/>
-      <c r="I25" s="163"/>
-      <c r="J25" s="163"/>
-      <c r="K25" s="163"/>
-      <c r="L25" s="163"/>
+      <c r="C25" s="154"/>
+      <c r="D25" s="154"/>
+      <c r="E25" s="154"/>
+      <c r="F25" s="154"/>
+      <c r="G25" s="154"/>
+      <c r="H25" s="154"/>
+      <c r="I25" s="154"/>
+      <c r="J25" s="154"/>
+      <c r="K25" s="154"/>
+      <c r="L25" s="154"/>
       <c r="M25" s="14"/>
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
     </row>
     <row r="26" spans="2:15" ht="30">
-      <c r="B26" s="161" t="s">
+      <c r="B26" s="152" t="s">
         <v>95</v>
       </c>
-      <c r="C26" s="162"/>
+      <c r="C26" s="153"/>
       <c r="D26" s="83"/>
       <c r="E26" s="80" t="s">
         <v>19</v>
@@ -3893,10 +3900,10 @@
       <c r="O26" s="6"/>
     </row>
     <row r="27" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B27" s="137" t="s">
+      <c r="B27" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C27" s="152"/>
+      <c r="C27" s="142"/>
       <c r="D27" s="76" t="s">
         <v>98</v>
       </c>
@@ -3921,7 +3928,7 @@
       <c r="K27" s="79">
         <v>0</v>
       </c>
-      <c r="L27" s="154">
+      <c r="L27" s="145">
         <f>(E27*E28)+(F27*F28)+(G27*G28)+(H27*H28)+(I27*I28)+(J27*J28)+(K27*K28)</f>
         <v>0</v>
       </c>
@@ -3930,8 +3937,8 @@
       <c r="O27" s="5"/>
     </row>
     <row r="28" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B28" s="139"/>
-      <c r="C28" s="153"/>
+      <c r="B28" s="147"/>
+      <c r="C28" s="148"/>
       <c r="D28" s="76" t="s">
         <v>99</v>
       </c>
@@ -3956,16 +3963,16 @@
       <c r="K28" s="74">
         <v>0</v>
       </c>
-      <c r="L28" s="155"/>
+      <c r="L28" s="146"/>
       <c r="M28" s="17"/>
       <c r="N28" s="5"/>
       <c r="O28" s="5"/>
     </row>
     <row r="29" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B29" s="137" t="s">
+      <c r="B29" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C29" s="152"/>
+      <c r="C29" s="142"/>
       <c r="D29" s="76" t="s">
         <v>98</v>
       </c>
@@ -3990,7 +3997,7 @@
       <c r="K29" s="79">
         <v>0</v>
       </c>
-      <c r="L29" s="154">
+      <c r="L29" s="145">
         <f>(E29*E30)+(F29*F30)+(G29*G30)+(H29*H30)+(I29*I30)+(J29*J30)+(K29*K30)</f>
         <v>0</v>
       </c>
@@ -3999,8 +4006,8 @@
       <c r="O29" s="5"/>
     </row>
     <row r="30" spans="2:15" ht="16.5" customHeight="1">
-      <c r="B30" s="139"/>
-      <c r="C30" s="153"/>
+      <c r="B30" s="147"/>
+      <c r="C30" s="148"/>
       <c r="D30" s="76" t="s">
         <v>99</v>
       </c>
@@ -4025,15 +4032,15 @@
       <c r="K30" s="74">
         <v>0</v>
       </c>
-      <c r="L30" s="155"/>
+      <c r="L30" s="146"/>
       <c r="M30" s="17"/>
       <c r="O30" s="5"/>
     </row>
     <row r="31" spans="2:15" ht="16.5" customHeight="1">
-      <c r="B31" s="137" t="s">
+      <c r="B31" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C31" s="152"/>
+      <c r="C31" s="142"/>
       <c r="D31" s="76" t="s">
         <v>98</v>
       </c>
@@ -4058,7 +4065,7 @@
       <c r="K31" s="79">
         <v>0</v>
       </c>
-      <c r="L31" s="154">
+      <c r="L31" s="145">
         <f>(E31*E32)+(F31*F32)+(G31*G32)+(H31*H32)+(I31*I32)+(J31*J32)+(K31*K32)</f>
         <v>0</v>
       </c>
@@ -4066,8 +4073,8 @@
       <c r="O31" s="5"/>
     </row>
     <row r="32" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B32" s="139"/>
-      <c r="C32" s="153"/>
+      <c r="B32" s="147"/>
+      <c r="C32" s="148"/>
       <c r="D32" s="76" t="s">
         <v>99</v>
       </c>
@@ -4092,16 +4099,16 @@
       <c r="K32" s="74">
         <v>0</v>
       </c>
-      <c r="L32" s="155"/>
+      <c r="L32" s="146"/>
       <c r="M32" s="17"/>
       <c r="N32" s="5"/>
       <c r="O32" s="5"/>
     </row>
     <row r="33" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B33" s="137" t="s">
+      <c r="B33" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C33" s="152"/>
+      <c r="C33" s="142"/>
       <c r="D33" s="76" t="s">
         <v>98</v>
       </c>
@@ -4126,7 +4133,7 @@
       <c r="K33" s="79">
         <v>0</v>
       </c>
-      <c r="L33" s="154">
+      <c r="L33" s="145">
         <f>(E33*E34)+(F33*F34)+(G33*G34)+(H33*H34)+(I33*I34)+(J33*J34)+(K33*K34)</f>
         <v>0</v>
       </c>
@@ -4135,8 +4142,8 @@
       <c r="O33" s="5"/>
     </row>
     <row r="34" spans="2:15" ht="16.5" customHeight="1">
-      <c r="B34" s="159"/>
-      <c r="C34" s="160"/>
+      <c r="B34" s="143"/>
+      <c r="C34" s="144"/>
       <c r="D34" s="84" t="s">
         <v>99</v>
       </c>
@@ -4161,15 +4168,15 @@
       <c r="K34" s="74">
         <v>0</v>
       </c>
-      <c r="L34" s="155"/>
+      <c r="L34" s="146"/>
       <c r="M34" s="17"/>
       <c r="O34" s="5"/>
     </row>
     <row r="35" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B35" s="137" t="s">
+      <c r="B35" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C35" s="152"/>
+      <c r="C35" s="142"/>
       <c r="D35" s="76" t="s">
         <v>98</v>
       </c>
@@ -4194,7 +4201,7 @@
       <c r="K35" s="79">
         <v>0</v>
       </c>
-      <c r="L35" s="154">
+      <c r="L35" s="145">
         <f>(E35*E36)+(F35*F36)+(G35*G36)+(H35*H36)+(I35*I36)+(J35*J36)+(K35*K36)</f>
         <v>0</v>
       </c>
@@ -4203,8 +4210,8 @@
       <c r="O35" s="5"/>
     </row>
     <row r="36" spans="2:15" ht="16.5" customHeight="1">
-      <c r="B36" s="159"/>
-      <c r="C36" s="160"/>
+      <c r="B36" s="143"/>
+      <c r="C36" s="144"/>
       <c r="D36" s="84" t="s">
         <v>99</v>
       </c>
@@ -4229,15 +4236,15 @@
       <c r="K36" s="74">
         <v>0</v>
       </c>
-      <c r="L36" s="155"/>
+      <c r="L36" s="146"/>
       <c r="M36" s="17"/>
       <c r="O36" s="5"/>
     </row>
     <row r="37" spans="2:15" ht="17.25" customHeight="1">
-      <c r="B37" s="137" t="s">
+      <c r="B37" s="141" t="s">
         <v>97</v>
       </c>
-      <c r="C37" s="152"/>
+      <c r="C37" s="142"/>
       <c r="D37" s="76" t="s">
         <v>98</v>
       </c>
@@ -4262,7 +4269,7 @@
       <c r="K37" s="79">
         <v>0</v>
       </c>
-      <c r="L37" s="154">
+      <c r="L37" s="145">
         <f>(E37*E38)+(F37*F38)+(G37*G38)+(H37*H38)+(I37*I38)+(J37*J38)+(K37*K38)</f>
         <v>0</v>
       </c>
@@ -4271,8 +4278,8 @@
       <c r="O37" s="5"/>
     </row>
     <row r="38" spans="2:15" ht="16.5" customHeight="1">
-      <c r="B38" s="159"/>
-      <c r="C38" s="160"/>
+      <c r="B38" s="143"/>
+      <c r="C38" s="144"/>
       <c r="D38" s="84" t="s">
         <v>99</v>
       </c>
@@ -4297,28 +4304,28 @@
       <c r="K38" s="74">
         <v>0</v>
       </c>
-      <c r="L38" s="155"/>
+      <c r="L38" s="146"/>
       <c r="M38" s="17"/>
       <c r="O38" s="5"/>
     </row>
     <row r="39" spans="2:15" ht="22.5" customHeight="1">
-      <c r="B39" s="167" t="s">
+      <c r="B39" s="140" t="s">
         <v>72</v>
       </c>
-      <c r="C39" s="167"/>
-      <c r="D39" s="167"/>
-      <c r="E39" s="167"/>
-      <c r="F39" s="167"/>
+      <c r="C39" s="140"/>
+      <c r="D39" s="140"/>
+      <c r="E39" s="140"/>
+      <c r="F39" s="140"/>
       <c r="G39" s="93">
         <f>IFERROR(AVERAGEIF(E23:K23, "&gt;0"), 0)</f>
         <v>0</v>
       </c>
-      <c r="H39" s="164" t="s">
+      <c r="H39" s="137" t="s">
         <v>100</v>
       </c>
-      <c r="I39" s="165"/>
-      <c r="J39" s="165"/>
-      <c r="K39" s="166"/>
+      <c r="I39" s="138"/>
+      <c r="J39" s="138"/>
+      <c r="K39" s="139"/>
       <c r="L39" s="86">
         <f>L23+L27+L29+L31+L33</f>
         <v>0</v>
@@ -4332,12 +4339,25 @@
     <protectedRange password="C6E9" sqref="B7:C22 B27:C38 E10:K10 E12:K12 E14:K14 E16:K16 E18:K18 E20:K20 E22:K22 E8:K8 E27:K38" name="Rango1"/>
   </protectedRanges>
   <mergeCells count="36">
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="B35:C36"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="B37:C38"/>
-    <mergeCell ref="L37:L38"/>
+    <mergeCell ref="B13:C14"/>
+    <mergeCell ref="B17:C18"/>
+    <mergeCell ref="B19:C20"/>
+    <mergeCell ref="B21:C22"/>
+    <mergeCell ref="B15:C16"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B7:C8"/>
+    <mergeCell ref="B9:C10"/>
+    <mergeCell ref="B11:C12"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="B6:D6"/>
     <mergeCell ref="B29:C30"/>
     <mergeCell ref="B31:C32"/>
     <mergeCell ref="L33:L34"/>
@@ -4349,25 +4369,12 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C28"/>
     <mergeCell ref="B25:L25"/>
-    <mergeCell ref="B4:L4"/>
-    <mergeCell ref="B5:L5"/>
-    <mergeCell ref="B7:C8"/>
-    <mergeCell ref="B9:C10"/>
-    <mergeCell ref="B11:C12"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="B13:C14"/>
-    <mergeCell ref="B17:C18"/>
-    <mergeCell ref="B19:C20"/>
-    <mergeCell ref="B21:C22"/>
-    <mergeCell ref="B15:C16"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B35:C36"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="B37:C38"/>
+    <mergeCell ref="L37:L38"/>
   </mergeCells>
   <phoneticPr fontId="31" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -4385,7 +4392,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:O99"/>
+  <dimension ref="B1:O100"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.3984375" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -4443,17 +4450,17 @@
       <c r="M3" s="6"/>
     </row>
     <row r="4" spans="2:15" ht="22.5" customHeight="1">
-      <c r="B4" s="168" t="s">
+      <c r="B4" s="218" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="168"/>
-      <c r="D4" s="168"/>
-      <c r="E4" s="168"/>
-      <c r="F4" s="168"/>
-      <c r="G4" s="168"/>
-      <c r="H4" s="168"/>
-      <c r="I4" s="168"/>
-      <c r="J4" s="168"/>
+      <c r="C4" s="218"/>
+      <c r="D4" s="218"/>
+      <c r="E4" s="218"/>
+      <c r="F4" s="218"/>
+      <c r="G4" s="218"/>
+      <c r="H4" s="218"/>
+      <c r="I4" s="218"/>
+      <c r="J4" s="218"/>
       <c r="K4" s="33"/>
       <c r="L4" s="33"/>
       <c r="M4" s="33"/>
@@ -4771,32 +4778,32 @@
       </c>
     </row>
     <row r="17" spans="2:10" ht="21.75" customHeight="1" thickBot="1">
-      <c r="B17" s="168" t="s">
+      <c r="B17" s="218" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="168"/>
-      <c r="D17" s="168"/>
-      <c r="E17" s="168"/>
-      <c r="F17" s="168"/>
-      <c r="G17" s="168"/>
-      <c r="H17" s="168"/>
-      <c r="I17" s="168"/>
-      <c r="J17" s="168"/>
+      <c r="C17" s="218"/>
+      <c r="D17" s="218"/>
+      <c r="E17" s="218"/>
+      <c r="F17" s="218"/>
+      <c r="G17" s="218"/>
+      <c r="H17" s="218"/>
+      <c r="I17" s="218"/>
+      <c r="J17" s="218"/>
     </row>
     <row r="18" spans="2:10" ht="29" thickBot="1">
       <c r="B18" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="169" t="s">
+      <c r="C18" s="219" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="170"/>
-      <c r="E18" s="171"/>
-      <c r="F18" s="181" t="s">
+      <c r="D18" s="220"/>
+      <c r="E18" s="221"/>
+      <c r="F18" s="231" t="s">
         <v>41</v>
       </c>
-      <c r="G18" s="182"/>
-      <c r="H18" s="183"/>
+      <c r="G18" s="232"/>
+      <c r="H18" s="233"/>
       <c r="I18" s="52" t="s">
         <v>40</v>
       </c>
@@ -4806,185 +4813,185 @@
     </row>
     <row r="19" spans="2:10" ht="32" customHeight="1">
       <c r="B19" s="112"/>
-      <c r="C19" s="172"/>
-      <c r="D19" s="173"/>
-      <c r="E19" s="174"/>
-      <c r="F19" s="172"/>
-      <c r="G19" s="173"/>
-      <c r="H19" s="174"/>
+      <c r="C19" s="222"/>
+      <c r="D19" s="223"/>
+      <c r="E19" s="224"/>
+      <c r="F19" s="222"/>
+      <c r="G19" s="223"/>
+      <c r="H19" s="224"/>
       <c r="I19" s="113"/>
       <c r="J19" s="114"/>
     </row>
     <row r="20" spans="2:10" ht="32" customHeight="1">
       <c r="B20" s="115"/>
-      <c r="C20" s="178"/>
-      <c r="D20" s="179"/>
-      <c r="E20" s="180"/>
-      <c r="F20" s="178"/>
-      <c r="G20" s="179"/>
-      <c r="H20" s="180"/>
+      <c r="C20" s="228"/>
+      <c r="D20" s="229"/>
+      <c r="E20" s="230"/>
+      <c r="F20" s="228"/>
+      <c r="G20" s="229"/>
+      <c r="H20" s="230"/>
       <c r="I20" s="116"/>
       <c r="J20" s="117"/>
     </row>
     <row r="21" spans="2:10" ht="32" customHeight="1" thickBot="1">
       <c r="B21" s="118"/>
-      <c r="C21" s="175"/>
-      <c r="D21" s="176"/>
-      <c r="E21" s="177"/>
-      <c r="F21" s="175"/>
-      <c r="G21" s="176"/>
-      <c r="H21" s="177"/>
+      <c r="C21" s="225"/>
+      <c r="D21" s="226"/>
+      <c r="E21" s="227"/>
+      <c r="F21" s="225"/>
+      <c r="G21" s="226"/>
+      <c r="H21" s="227"/>
       <c r="I21" s="119"/>
       <c r="J21" s="120"/>
     </row>
     <row r="22" spans="2:10" ht="14" thickBot="1"/>
     <row r="23" spans="2:10" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B23" s="187" t="s">
+      <c r="B23" s="208" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="188"/>
-      <c r="D23" s="188"/>
-      <c r="E23" s="189"/>
-      <c r="F23" s="187" t="s">
+      <c r="C23" s="209"/>
+      <c r="D23" s="209"/>
+      <c r="E23" s="210"/>
+      <c r="F23" s="208" t="s">
         <v>44</v>
       </c>
-      <c r="G23" s="188"/>
-      <c r="H23" s="188"/>
-      <c r="I23" s="188"/>
-      <c r="J23" s="189"/>
+      <c r="G23" s="209"/>
+      <c r="H23" s="209"/>
+      <c r="I23" s="209"/>
+      <c r="J23" s="210"/>
     </row>
     <row r="24" spans="2:10" ht="18.75" customHeight="1">
-      <c r="B24" s="190" t="s">
+      <c r="B24" s="211" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="191"/>
-      <c r="D24" s="191"/>
-      <c r="E24" s="191"/>
-      <c r="F24" s="194" t="s">
+      <c r="C24" s="212"/>
+      <c r="D24" s="212"/>
+      <c r="E24" s="212"/>
+      <c r="F24" s="217" t="s">
         <v>53</v>
       </c>
-      <c r="G24" s="194"/>
-      <c r="H24" s="194"/>
-      <c r="I24" s="194"/>
-      <c r="J24" s="194"/>
+      <c r="G24" s="217"/>
+      <c r="H24" s="217"/>
+      <c r="I24" s="217"/>
+      <c r="J24" s="217"/>
     </row>
     <row r="25" spans="2:10" ht="22.5" customHeight="1">
-      <c r="B25" s="192" t="s">
+      <c r="B25" s="213" t="s">
         <v>46</v>
       </c>
-      <c r="C25" s="193"/>
-      <c r="D25" s="193"/>
-      <c r="E25" s="193"/>
-      <c r="F25" s="184" t="s">
+      <c r="C25" s="214"/>
+      <c r="D25" s="214"/>
+      <c r="E25" s="214"/>
+      <c r="F25" s="204" t="s">
         <v>54</v>
       </c>
-      <c r="G25" s="184"/>
-      <c r="H25" s="184"/>
-      <c r="I25" s="184"/>
-      <c r="J25" s="184"/>
+      <c r="G25" s="204"/>
+      <c r="H25" s="204"/>
+      <c r="I25" s="204"/>
+      <c r="J25" s="204"/>
     </row>
     <row r="26" spans="2:10" ht="21" customHeight="1">
-      <c r="B26" s="185" t="s">
+      <c r="B26" s="215" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="186"/>
-      <c r="D26" s="186"/>
-      <c r="E26" s="186"/>
-      <c r="F26" s="184" t="s">
+      <c r="C26" s="216"/>
+      <c r="D26" s="216"/>
+      <c r="E26" s="216"/>
+      <c r="F26" s="204" t="s">
         <v>55</v>
       </c>
-      <c r="G26" s="184"/>
-      <c r="H26" s="184"/>
-      <c r="I26" s="184"/>
-      <c r="J26" s="184"/>
+      <c r="G26" s="204"/>
+      <c r="H26" s="204"/>
+      <c r="I26" s="204"/>
+      <c r="J26" s="204"/>
     </row>
     <row r="27" spans="2:10" ht="21.75" customHeight="1">
-      <c r="B27" s="185" t="s">
+      <c r="B27" s="215" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="186"/>
-      <c r="D27" s="186"/>
-      <c r="E27" s="186"/>
-      <c r="F27" s="184" t="s">
+      <c r="C27" s="216"/>
+      <c r="D27" s="216"/>
+      <c r="E27" s="216"/>
+      <c r="F27" s="204" t="s">
         <v>56</v>
       </c>
-      <c r="G27" s="184"/>
-      <c r="H27" s="184"/>
-      <c r="I27" s="184"/>
-      <c r="J27" s="184"/>
+      <c r="G27" s="204"/>
+      <c r="H27" s="204"/>
+      <c r="I27" s="204"/>
+      <c r="J27" s="204"/>
     </row>
     <row r="28" spans="2:10" ht="20.25" customHeight="1">
-      <c r="B28" s="185" t="s">
+      <c r="B28" s="215" t="s">
         <v>49</v>
       </c>
-      <c r="C28" s="186"/>
-      <c r="D28" s="186"/>
-      <c r="E28" s="186"/>
-      <c r="F28" s="184" t="s">
+      <c r="C28" s="216"/>
+      <c r="D28" s="216"/>
+      <c r="E28" s="216"/>
+      <c r="F28" s="204" t="s">
         <v>57</v>
       </c>
-      <c r="G28" s="184"/>
-      <c r="H28" s="184"/>
-      <c r="I28" s="184"/>
-      <c r="J28" s="184"/>
+      <c r="G28" s="204"/>
+      <c r="H28" s="204"/>
+      <c r="I28" s="204"/>
+      <c r="J28" s="204"/>
     </row>
     <row r="29" spans="2:10" ht="24" customHeight="1">
-      <c r="B29" s="185" t="s">
+      <c r="B29" s="215" t="s">
         <v>50</v>
       </c>
-      <c r="C29" s="186"/>
-      <c r="D29" s="186"/>
-      <c r="E29" s="186"/>
-      <c r="F29" s="184" t="s">
+      <c r="C29" s="216"/>
+      <c r="D29" s="216"/>
+      <c r="E29" s="216"/>
+      <c r="F29" s="204" t="s">
         <v>58</v>
       </c>
-      <c r="G29" s="184"/>
-      <c r="H29" s="184"/>
-      <c r="I29" s="184"/>
-      <c r="J29" s="184"/>
+      <c r="G29" s="204"/>
+      <c r="H29" s="204"/>
+      <c r="I29" s="204"/>
+      <c r="J29" s="204"/>
     </row>
     <row r="30" spans="2:10" ht="20.25" customHeight="1">
-      <c r="B30" s="185" t="s">
+      <c r="B30" s="215" t="s">
         <v>51</v>
       </c>
-      <c r="C30" s="186"/>
-      <c r="D30" s="186"/>
-      <c r="E30" s="186"/>
-      <c r="F30" s="184" t="s">
+      <c r="C30" s="216"/>
+      <c r="D30" s="216"/>
+      <c r="E30" s="216"/>
+      <c r="F30" s="204" t="s">
         <v>59</v>
       </c>
-      <c r="G30" s="184"/>
-      <c r="H30" s="184"/>
-      <c r="I30" s="184"/>
-      <c r="J30" s="184"/>
+      <c r="G30" s="204"/>
+      <c r="H30" s="204"/>
+      <c r="I30" s="204"/>
+      <c r="J30" s="204"/>
     </row>
     <row r="31" spans="2:10" ht="19.5" customHeight="1">
-      <c r="B31" s="185" t="s">
+      <c r="B31" s="215" t="s">
         <v>52</v>
       </c>
-      <c r="C31" s="186"/>
-      <c r="D31" s="186"/>
-      <c r="E31" s="186"/>
-      <c r="F31" s="184" t="s">
+      <c r="C31" s="216"/>
+      <c r="D31" s="216"/>
+      <c r="E31" s="216"/>
+      <c r="F31" s="204" t="s">
         <v>60</v>
       </c>
-      <c r="G31" s="184"/>
-      <c r="H31" s="184"/>
-      <c r="I31" s="184"/>
-      <c r="J31" s="184"/>
+      <c r="G31" s="204"/>
+      <c r="H31" s="204"/>
+      <c r="I31" s="204"/>
+      <c r="J31" s="204"/>
     </row>
     <row r="33" spans="2:10" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B33" s="195" t="s">
+      <c r="B33" s="205" t="s">
         <v>61</v>
       </c>
-      <c r="C33" s="196"/>
-      <c r="D33" s="196"/>
-      <c r="E33" s="196"/>
-      <c r="F33" s="196"/>
-      <c r="G33" s="196"/>
-      <c r="H33" s="196"/>
-      <c r="I33" s="196"/>
-      <c r="J33" s="197"/>
+      <c r="C33" s="206"/>
+      <c r="D33" s="206"/>
+      <c r="E33" s="206"/>
+      <c r="F33" s="206"/>
+      <c r="G33" s="206"/>
+      <c r="H33" s="206"/>
+      <c r="I33" s="206"/>
+      <c r="J33" s="207"/>
     </row>
     <row r="34" spans="2:10" ht="78" customHeight="1">
       <c r="B34" s="56" t="s">
@@ -5263,165 +5270,173 @@
     </row>
     <row r="45" spans="2:10" ht="24" customHeight="1">
       <c r="B45" s="68"/>
-      <c r="C45" s="198" t="s">
+      <c r="C45" s="169" t="s">
         <v>75</v>
       </c>
-      <c r="D45" s="198"/>
-      <c r="E45" s="198"/>
-      <c r="F45" s="198"/>
-      <c r="G45" s="198"/>
-      <c r="H45" s="198"/>
+      <c r="D45" s="169"/>
+      <c r="E45" s="169"/>
+      <c r="F45" s="169"/>
+      <c r="G45" s="169"/>
+      <c r="H45" s="169"/>
       <c r="I45" s="67"/>
       <c r="J45" s="67"/>
     </row>
-    <row r="46" spans="2:10" ht="56.25" customHeight="1">
-      <c r="B46" s="199" t="s">
+    <row r="46" spans="2:10" ht="39" customHeight="1">
+      <c r="B46" s="203" t="s">
         <v>74</v>
       </c>
-      <c r="C46" s="199"/>
-      <c r="D46" s="199"/>
+      <c r="C46" s="203"/>
+      <c r="D46" s="203"/>
       <c r="E46" s="96">
         <v>0</v>
       </c>
-      <c r="F46" s="199" t="s">
+      <c r="F46" s="203" t="s">
         <v>73</v>
       </c>
-      <c r="G46" s="199"/>
-      <c r="H46" s="199"/>
-      <c r="I46" s="199"/>
+      <c r="G46" s="203"/>
+      <c r="H46" s="203"/>
+      <c r="I46" s="203"/>
       <c r="J46" s="95">
         <f>'Table 2'!L39</f>
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:10" ht="42" customHeight="1">
-      <c r="B47" s="199" t="s">
+    <row r="47" spans="2:10" ht="39" customHeight="1">
+      <c r="B47" s="203" t="s">
         <v>76</v>
       </c>
-      <c r="C47" s="199"/>
-      <c r="D47" s="199"/>
+      <c r="C47" s="203"/>
+      <c r="D47" s="203"/>
       <c r="E47" s="94">
         <f>E46+J46</f>
         <v>0</v>
       </c>
-      <c r="F47" s="203" t="s">
+      <c r="F47" s="200" t="s">
         <v>77</v>
       </c>
-      <c r="G47" s="204"/>
-      <c r="H47" s="204"/>
-      <c r="I47" s="205"/>
+      <c r="G47" s="201"/>
+      <c r="H47" s="201"/>
+      <c r="I47" s="202"/>
       <c r="J47" s="92">
         <f>'Table 2'!G39</f>
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:10" ht="47.25" customHeight="1">
-      <c r="B48" s="199" t="s">
+    <row r="48" spans="2:10" ht="39" customHeight="1">
+      <c r="B48" s="203" t="s">
         <v>78</v>
       </c>
-      <c r="C48" s="199"/>
-      <c r="D48" s="199"/>
+      <c r="C48" s="203"/>
+      <c r="D48" s="203"/>
       <c r="E48" s="97">
         <v>0</v>
       </c>
-      <c r="F48" s="203" t="s">
+      <c r="F48" s="200" t="s">
         <v>79</v>
       </c>
-      <c r="G48" s="204"/>
-      <c r="H48" s="204"/>
-      <c r="I48" s="205"/>
+      <c r="G48" s="201"/>
+      <c r="H48" s="201"/>
+      <c r="I48" s="202"/>
       <c r="J48" s="92">
         <f>((J47*5)/60)*6</f>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:10" ht="32.25" customHeight="1">
-      <c r="B49" s="199" t="s">
+    <row r="49" spans="2:10" s="234" customFormat="1" ht="39" customHeight="1">
+      <c r="B49" s="200" t="s">
+        <v>109</v>
+      </c>
+      <c r="C49" s="201"/>
+      <c r="D49" s="202"/>
+      <c r="E49" s="97">
+        <v>0</v>
+      </c>
+      <c r="F49" s="200" t="s">
+        <v>110</v>
+      </c>
+      <c r="G49" s="201"/>
+      <c r="H49" s="201"/>
+      <c r="I49" s="202"/>
+      <c r="J49" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" ht="32.25" customHeight="1">
+      <c r="B50" s="203" t="s">
         <v>80</v>
       </c>
-      <c r="C49" s="199"/>
-      <c r="D49" s="199"/>
-      <c r="E49" s="97">
-        <v>0</v>
-      </c>
-      <c r="F49" s="203" t="s">
+      <c r="C50" s="203"/>
+      <c r="D50" s="203"/>
+      <c r="E50" s="97">
+        <v>0</v>
+      </c>
+      <c r="F50" s="200" t="s">
         <v>81</v>
       </c>
-      <c r="G49" s="204"/>
-      <c r="H49" s="204"/>
-      <c r="I49" s="205"/>
-      <c r="J49" s="98">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="2:10" ht="40.5" customHeight="1">
-      <c r="B50" s="200" t="s">
+      <c r="G50" s="201"/>
+      <c r="H50" s="201"/>
+      <c r="I50" s="202"/>
+      <c r="J50" s="98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" ht="40.5" customHeight="1">
+      <c r="B51" s="197" t="s">
         <v>82</v>
       </c>
-      <c r="C50" s="200"/>
-      <c r="D50" s="69">
-        <v>0</v>
-      </c>
-      <c r="E50" s="89" t="s">
+      <c r="C51" s="197"/>
+      <c r="D51" s="69">
+        <v>0</v>
+      </c>
+      <c r="E51" s="89" t="s">
         <v>83</v>
       </c>
-      <c r="F50" s="200" t="s">
+      <c r="F51" s="197" t="s">
         <v>85</v>
       </c>
-      <c r="G50" s="200"/>
-      <c r="H50" s="91">
-        <v>0</v>
-      </c>
-      <c r="I50" s="201" t="s">
+      <c r="G51" s="197"/>
+      <c r="H51" s="91">
+        <v>0</v>
+      </c>
+      <c r="I51" s="198" t="s">
         <v>83</v>
       </c>
-      <c r="J50" s="201"/>
-    </row>
-    <row r="51" spans="2:10" ht="30.75" customHeight="1">
-      <c r="B51" s="200"/>
-      <c r="C51" s="200"/>
-      <c r="D51" s="69">
-        <v>0</v>
-      </c>
-      <c r="E51" s="90" t="s">
+      <c r="J51" s="198"/>
+    </row>
+    <row r="52" spans="2:10" ht="30.75" customHeight="1">
+      <c r="B52" s="197"/>
+      <c r="C52" s="197"/>
+      <c r="D52" s="69">
+        <v>0</v>
+      </c>
+      <c r="E52" s="90" t="s">
         <v>84</v>
       </c>
-      <c r="F51" s="200"/>
-      <c r="G51" s="200"/>
-      <c r="H51" s="91">
-        <v>0</v>
-      </c>
-      <c r="I51" s="202" t="s">
+      <c r="F52" s="197"/>
+      <c r="G52" s="197"/>
+      <c r="H52" s="91">
+        <v>0</v>
+      </c>
+      <c r="I52" s="199" t="s">
         <v>86</v>
       </c>
-      <c r="J51" s="202"/>
-    </row>
-    <row r="54" spans="2:10" ht="27.75" customHeight="1">
-      <c r="B54" s="198" t="s">
+      <c r="J52" s="199"/>
+    </row>
+    <row r="55" spans="2:10" ht="27.75" customHeight="1">
+      <c r="B55" s="169" t="s">
         <v>87</v>
       </c>
-      <c r="C54" s="198"/>
-      <c r="D54" s="198"/>
-      <c r="E54" s="198"/>
-      <c r="F54" s="198"/>
-      <c r="G54" s="198"/>
-      <c r="H54" s="198"/>
-      <c r="I54" s="198"/>
-      <c r="J54" s="198"/>
-    </row>
-    <row r="59" spans="2:10" ht="24" customHeight="1"/>
-    <row r="77" ht="20" customHeight="1"/>
-    <row r="86" spans="2:10">
-      <c r="B86" s="12"/>
-      <c r="C86" s="12"/>
-      <c r="D86" s="12"/>
-      <c r="E86" s="12"/>
-      <c r="F86" s="12"/>
-      <c r="G86" s="12"/>
-      <c r="H86" s="12"/>
-      <c r="I86" s="12"/>
-      <c r="J86" s="12"/>
-    </row>
+      <c r="C55" s="169"/>
+      <c r="D55" s="169"/>
+      <c r="E55" s="169"/>
+      <c r="F55" s="169"/>
+      <c r="G55" s="169"/>
+      <c r="H55" s="169"/>
+      <c r="I55" s="169"/>
+      <c r="J55" s="169"/>
+    </row>
+    <row r="60" spans="2:10" ht="24" customHeight="1"/>
+    <row r="78" ht="20" customHeight="1"/>
     <row r="87" spans="2:10">
       <c r="B87" s="12"/>
       <c r="C87" s="12"/>
@@ -5489,120 +5504,85 @@
       <c r="J92" s="12"/>
     </row>
     <row r="93" spans="2:10">
-      <c r="B93" s="228"/>
-      <c r="C93" s="224"/>
-      <c r="D93" s="225"/>
-      <c r="E93" s="220"/>
-      <c r="F93" s="221"/>
-      <c r="G93" s="219"/>
-      <c r="H93" s="219"/>
-      <c r="I93" s="213"/>
-      <c r="J93" s="214"/>
-    </row>
-    <row r="94" spans="2:10" ht="50" customHeight="1">
-      <c r="B94" s="229"/>
-      <c r="C94" s="226"/>
-      <c r="D94" s="227"/>
-      <c r="E94" s="222"/>
-      <c r="F94" s="223"/>
-      <c r="G94" s="219"/>
-      <c r="H94" s="219"/>
-      <c r="I94" s="215"/>
-      <c r="J94" s="216"/>
-    </row>
-    <row r="95" spans="2:10" ht="32.25" customHeight="1">
-      <c r="B95" s="10"/>
-      <c r="C95" s="230"/>
-      <c r="D95" s="231"/>
-      <c r="E95" s="207"/>
-      <c r="F95" s="208"/>
-      <c r="G95" s="217"/>
-      <c r="H95" s="217"/>
-      <c r="I95" s="211"/>
-      <c r="J95" s="212"/>
-    </row>
-    <row r="96" spans="2:10" ht="30">
-      <c r="B96" s="99" t="s">
+      <c r="B93" s="12"/>
+      <c r="C93" s="12"/>
+      <c r="D93" s="12"/>
+      <c r="E93" s="12"/>
+      <c r="F93" s="12"/>
+      <c r="G93" s="12"/>
+      <c r="H93" s="12"/>
+      <c r="I93" s="12"/>
+      <c r="J93" s="12"/>
+    </row>
+    <row r="94" spans="2:10">
+      <c r="B94" s="191"/>
+      <c r="C94" s="187"/>
+      <c r="D94" s="188"/>
+      <c r="E94" s="183"/>
+      <c r="F94" s="184"/>
+      <c r="G94" s="182"/>
+      <c r="H94" s="182"/>
+      <c r="I94" s="176"/>
+      <c r="J94" s="177"/>
+    </row>
+    <row r="95" spans="2:10" ht="50" customHeight="1">
+      <c r="B95" s="192"/>
+      <c r="C95" s="189"/>
+      <c r="D95" s="190"/>
+      <c r="E95" s="185"/>
+      <c r="F95" s="186"/>
+      <c r="G95" s="182"/>
+      <c r="H95" s="182"/>
+      <c r="I95" s="178"/>
+      <c r="J95" s="179"/>
+    </row>
+    <row r="96" spans="2:10" ht="32.25" customHeight="1">
+      <c r="B96" s="10"/>
+      <c r="C96" s="193"/>
+      <c r="D96" s="194"/>
+      <c r="E96" s="170"/>
+      <c r="F96" s="171"/>
+      <c r="G96" s="180"/>
+      <c r="H96" s="180"/>
+      <c r="I96" s="174"/>
+      <c r="J96" s="175"/>
+    </row>
+    <row r="97" spans="2:10" ht="30">
+      <c r="B97" s="99" t="s">
         <v>102</v>
       </c>
-      <c r="C96" s="232" t="s">
+      <c r="C97" s="195" t="s">
         <v>91</v>
       </c>
-      <c r="D96" s="233"/>
-      <c r="E96" s="218" t="s">
+      <c r="D97" s="196"/>
+      <c r="E97" s="181" t="s">
         <v>90</v>
       </c>
-      <c r="F96" s="218"/>
-      <c r="G96" s="218" t="s">
+      <c r="F97" s="181"/>
+      <c r="G97" s="181" t="s">
         <v>89</v>
       </c>
-      <c r="H96" s="218"/>
-      <c r="I96" s="209" t="s">
+      <c r="H97" s="181"/>
+      <c r="I97" s="172" t="s">
         <v>88</v>
       </c>
-      <c r="J96" s="210"/>
-    </row>
-    <row r="99" spans="2:8">
-      <c r="B99" s="206"/>
-      <c r="C99" s="206"/>
-      <c r="D99" s="206"/>
-      <c r="E99" s="206"/>
-      <c r="F99" s="206"/>
-      <c r="G99" s="206"/>
-      <c r="H99" s="206"/>
+      <c r="J97" s="173"/>
+    </row>
+    <row r="100" spans="2:10">
+      <c r="B100" s="168"/>
+      <c r="C100" s="168"/>
+      <c r="D100" s="168"/>
+      <c r="E100" s="168"/>
+      <c r="F100" s="168"/>
+      <c r="G100" s="168"/>
+      <c r="H100" s="168"/>
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange algorithmName="SHA-512" hashValue="RErhUU0R46kti2op2YNumjcTMI2JuReaXJQBWF7UO/8PHK7o2wlWCLBFwJEJ/vjOrQzyuQwKslsoAy2D6y8uHA==" saltValue="LKhi+thnO+BACQ7B33xZFA==" spinCount="100000" sqref="C7:J13 B19:J21 E48:E49 J49 D50:D51 H50:H51 B95:C95 C35:J41" name="Rango1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="RErhUU0R46kti2op2YNumjcTMI2JuReaXJQBWF7UO/8PHK7o2wlWCLBFwJEJ/vjOrQzyuQwKslsoAy2D6y8uHA==" saltValue="LKhi+thnO+BACQ7B33xZFA==" spinCount="100000" sqref="C7:J13 B19:J21 E48 J50 D51:D52 H51:H52 B96:C96 C35:J41 E50" name="Rango1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="RErhUU0R46kti2op2YNumjcTMI2JuReaXJQBWF7UO/8PHK7o2wlWCLBFwJEJ/vjOrQzyuQwKslsoAy2D6y8uHA==" saltValue="LKhi+thnO+BACQ7B33xZFA==" spinCount="100000" sqref="E49" name="Rango1_1"/>
   </protectedRanges>
-  <mergeCells count="57">
-    <mergeCell ref="B99:H99"/>
-    <mergeCell ref="B54:J54"/>
-    <mergeCell ref="E95:F95"/>
-    <mergeCell ref="I96:J96"/>
-    <mergeCell ref="I95:J95"/>
-    <mergeCell ref="I93:J94"/>
-    <mergeCell ref="G95:H95"/>
-    <mergeCell ref="G96:H96"/>
-    <mergeCell ref="G93:H94"/>
-    <mergeCell ref="E96:F96"/>
-    <mergeCell ref="E93:F94"/>
-    <mergeCell ref="C93:D94"/>
-    <mergeCell ref="B93:B94"/>
-    <mergeCell ref="C95:D95"/>
-    <mergeCell ref="C96:D96"/>
-    <mergeCell ref="B50:C51"/>
-    <mergeCell ref="F50:G51"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="F31:J31"/>
-    <mergeCell ref="B33:J33"/>
-    <mergeCell ref="C45:H45"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="F23:J23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="F24:J24"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="F27:J27"/>
-    <mergeCell ref="F28:J28"/>
-    <mergeCell ref="F29:J29"/>
-    <mergeCell ref="F30:J30"/>
-    <mergeCell ref="F25:J25"/>
-    <mergeCell ref="F26:J26"/>
+  <mergeCells count="59">
     <mergeCell ref="B4:J4"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C19:E19"/>
@@ -5613,6 +5593,55 @@
     <mergeCell ref="F19:H19"/>
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="C21:E21"/>
+    <mergeCell ref="F27:J27"/>
+    <mergeCell ref="F28:J28"/>
+    <mergeCell ref="F29:J29"/>
+    <mergeCell ref="F30:J30"/>
+    <mergeCell ref="F25:J25"/>
+    <mergeCell ref="F26:J26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="F23:J23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="F24:J24"/>
+    <mergeCell ref="F31:J31"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="C45:H45"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="B51:C52"/>
+    <mergeCell ref="F51:G52"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="B100:H100"/>
+    <mergeCell ref="B55:J55"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="I97:J97"/>
+    <mergeCell ref="I96:J96"/>
+    <mergeCell ref="I94:J95"/>
+    <mergeCell ref="G96:H96"/>
+    <mergeCell ref="G97:H97"/>
+    <mergeCell ref="G94:H95"/>
+    <mergeCell ref="E97:F97"/>
+    <mergeCell ref="E94:F95"/>
+    <mergeCell ref="C94:D95"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="C96:D96"/>
+    <mergeCell ref="C97:D97"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -5623,8 +5652,8 @@
   <rowBreaks count="4" manualBreakCount="4">
     <brk id="22" max="16383" man="1"/>
     <brk id="32" max="16383" man="1"/>
-    <brk id="52" max="16383" man="1"/>
-    <brk id="92" max="10" man="1"/>
+    <brk id="52" max="10" man="1"/>
+    <brk id="93" max="10" man="1"/>
   </rowBreaks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>